<commit_message>
changes has been made
</commit_message>
<xml_diff>
--- a/test-results/withdraw_result.xlsx
+++ b/test-results/withdraw_result.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D8"/>
   <cols>
     <col min="1" max="1" width="27.83203125" customWidth="1"/>
     <col min="2" max="2" width="35.83203125" customWidth="1"/>
@@ -421,13 +421,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Network issue</v>
+        <v>Testing boundary case</v>
       </c>
       <c r="B2" t="str">
-        <v>10-Apr-2026 (09:00 AM - 06:00 PM)</v>
+        <v>02-Apr-2026 (10:00 AM - 07:00 PM)</v>
       </c>
       <c r="C2" t="str">
-        <v>Not Found</v>
+        <v>completed</v>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -435,10 +435,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Forgot to punch-out</v>
+        <v>Network issue</v>
       </c>
       <c r="B3" t="str">
-        <v>22-Apr-2026 07:30 PM</v>
+        <v>01-May-2026 (09:30 AM - 06:30 PM)</v>
       </c>
       <c r="C3" t="str">
         <v>completed</v>
@@ -449,10 +449,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Device was not working</v>
+        <v>Network issue</v>
       </c>
       <c r="B4" t="str">
-        <v>20-Apr-2026 11:00 AM</v>
+        <v>03-May-2026 (09:00 AM - 06:00 PM)</v>
       </c>
       <c r="C4" t="str">
         <v>completed</v>
@@ -463,13 +463,13 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>System was down whole day</v>
+        <v>Network issue</v>
       </c>
       <c r="B5" t="str">
-        <v>15-Apr-2026 (08:30 AM - 05:30 PM)</v>
+        <v>01-Apr-2026 (09:00 AM - 06:00 PM)</v>
       </c>
       <c r="C5" t="str">
-        <v>Not Found</v>
+        <v>completed</v>
       </c>
       <c r="D5" t="str">
         <v/>
@@ -477,21 +477,49 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
+        <v>System was down whole day</v>
+      </c>
+      <c r="B6" t="str">
+        <v>15-Apr-2026 (08:30 AM - 05:30 PM)</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Not Found</v>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
         <v>Network issue</v>
       </c>
-      <c r="B6" t="str">
+      <c r="B7" t="str">
         <v>16-Apr-2026 09:00 AM</v>
       </c>
-      <c r="C6" t="str">
+      <c r="C7" t="str">
+        <v>Not Found</v>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Network issue</v>
+      </c>
+      <c r="B8" t="str">
+        <v>02-May-2026 (09:30 AM - 06:30 PM)</v>
+      </c>
+      <c r="C8" t="str">
         <v>completed</v>
       </c>
-      <c r="D6" t="str">
+      <c r="D8" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>